<commit_message>
Monthly writing paper sales
</commit_message>
<xml_diff>
--- a/shatrov_bootstraps_res.xlsx
+++ b/shatrov_bootstraps_res.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Игорь\Desktop\sem_8\mipt_diplom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997BDE62-46C6-46C8-83B1-A37809988675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B0526A-92FE-4B67-9D1D-F981FFEF7C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Информация про ряды" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="32">
   <si>
     <t>Номер</t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>Отсутствует сезонность. Похож на сумму тренда и случайного блуждания</t>
+  </si>
+  <si>
+    <t>https://raw.githubusercontent.com/jbrownlee/Datasets/master/monthly-writing-paper-sales.csv</t>
+  </si>
+  <si>
+    <t>Monthly Writing Paper Sales</t>
   </si>
 </sst>
 </file>
@@ -128,7 +134,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -146,6 +152,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -180,27 +194,32 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Гиперссылка" xfId="1" builtinId="8"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -479,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D4:G8"/>
+  <dimension ref="D4:G9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="8.88671875" customWidth="1"/>
@@ -555,14 +574,31 @@
         <v>29</v>
       </c>
     </row>
+    <row r="9" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G9" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F9" r:id="rId1" xr:uid="{9367D316-61C7-4D04-93AD-9FDC62845A8C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5432242B-BB45-4574-A5B4-2CF25C9CDCFF}">
-  <dimension ref="D4:H40"/>
+  <dimension ref="D4:H49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="13.21875" customWidth="1"/>
@@ -584,7 +620,7 @@
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
       <c r="E5" t="s">
@@ -598,7 +634,7 @@
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D6" s="5"/>
+      <c r="D6" s="4"/>
       <c r="E6" t="s">
         <v>16</v>
       </c>
@@ -610,7 +646,7 @@
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D7" s="5"/>
+      <c r="D7" s="4"/>
       <c r="E7" t="s">
         <v>10</v>
       </c>
@@ -622,7 +658,7 @@
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D8" s="5"/>
+      <c r="D8" s="4"/>
       <c r="E8" t="s">
         <v>11</v>
       </c>
@@ -634,7 +670,7 @@
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D9" s="5"/>
+      <c r="D9" s="4"/>
       <c r="E9" t="s">
         <v>12</v>
       </c>
@@ -646,7 +682,7 @@
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D10" s="5"/>
+      <c r="D10" s="4"/>
       <c r="E10" t="s">
         <v>13</v>
       </c>
@@ -658,7 +694,7 @@
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D11" s="5"/>
+      <c r="D11" s="4"/>
       <c r="E11" t="s">
         <v>14</v>
       </c>
@@ -670,7 +706,7 @@
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D12" s="5"/>
+      <c r="D12" s="4"/>
       <c r="E12" t="s">
         <v>15</v>
       </c>
@@ -682,13 +718,13 @@
       </c>
     </row>
     <row r="13" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>2</v>
       </c>
       <c r="E14" t="s">
@@ -702,7 +738,7 @@
       </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D15" s="5"/>
+      <c r="D15" s="4"/>
       <c r="E15" t="s">
         <v>16</v>
       </c>
@@ -714,7 +750,7 @@
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D16" s="5"/>
+      <c r="D16" s="4"/>
       <c r="E16" t="s">
         <v>10</v>
       </c>
@@ -726,7 +762,7 @@
       </c>
     </row>
     <row r="17" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D17" s="5"/>
+      <c r="D17" s="4"/>
       <c r="E17" t="s">
         <v>11</v>
       </c>
@@ -738,7 +774,7 @@
       </c>
     </row>
     <row r="18" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D18" s="5"/>
+      <c r="D18" s="4"/>
       <c r="E18" t="s">
         <v>12</v>
       </c>
@@ -750,7 +786,7 @@
       </c>
     </row>
     <row r="19" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D19" s="5"/>
+      <c r="D19" s="4"/>
       <c r="E19" t="s">
         <v>13</v>
       </c>
@@ -762,7 +798,7 @@
       </c>
     </row>
     <row r="20" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D20" s="5"/>
+      <c r="D20" s="4"/>
       <c r="E20" t="s">
         <v>14</v>
       </c>
@@ -774,7 +810,7 @@
       </c>
     </row>
     <row r="21" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D21" s="5"/>
+      <c r="D21" s="4"/>
       <c r="E21" t="s">
         <v>15</v>
       </c>
@@ -786,13 +822,13 @@
       </c>
     </row>
     <row r="22" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
     </row>
     <row r="23" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D23" s="5">
+      <c r="D23" s="4">
         <v>3</v>
       </c>
       <c r="E23" t="s">
@@ -809,7 +845,7 @@
       </c>
     </row>
     <row r="24" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D24" s="5"/>
+      <c r="D24" s="4"/>
       <c r="E24" t="s">
         <v>16</v>
       </c>
@@ -821,7 +857,7 @@
       </c>
     </row>
     <row r="25" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D25" s="5"/>
+      <c r="D25" s="4"/>
       <c r="E25" t="s">
         <v>10</v>
       </c>
@@ -833,7 +869,7 @@
       </c>
     </row>
     <row r="26" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D26" s="5"/>
+      <c r="D26" s="4"/>
       <c r="E26" t="s">
         <v>11</v>
       </c>
@@ -845,7 +881,7 @@
       </c>
     </row>
     <row r="27" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D27" s="5"/>
+      <c r="D27" s="4"/>
       <c r="E27" t="s">
         <v>12</v>
       </c>
@@ -857,7 +893,7 @@
       </c>
     </row>
     <row r="28" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D28" s="5"/>
+      <c r="D28" s="4"/>
       <c r="E28" t="s">
         <v>13</v>
       </c>
@@ -869,7 +905,7 @@
       </c>
     </row>
     <row r="29" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D29" s="5"/>
+      <c r="D29" s="4"/>
       <c r="E29" t="s">
         <v>14</v>
       </c>
@@ -881,7 +917,7 @@
       </c>
     </row>
     <row r="30" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D30" s="5"/>
+      <c r="D30" s="4"/>
       <c r="E30" t="s">
         <v>15</v>
       </c>
@@ -893,13 +929,13 @@
       </c>
     </row>
     <row r="31" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
     </row>
     <row r="32" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D32" s="5">
+      <c r="D32" s="4">
         <v>4</v>
       </c>
       <c r="E32" t="s">
@@ -913,7 +949,7 @@
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D33" s="5"/>
+      <c r="D33" s="4"/>
       <c r="E33" t="s">
         <v>16</v>
       </c>
@@ -925,7 +961,7 @@
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D34" s="5"/>
+      <c r="D34" s="4"/>
       <c r="E34" t="s">
         <v>10</v>
       </c>
@@ -937,7 +973,7 @@
       </c>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D35" s="5"/>
+      <c r="D35" s="4"/>
       <c r="E35" t="s">
         <v>11</v>
       </c>
@@ -949,7 +985,7 @@
       </c>
     </row>
     <row r="36" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D36" s="5"/>
+      <c r="D36" s="4"/>
       <c r="E36" t="s">
         <v>12</v>
       </c>
@@ -961,7 +997,7 @@
       </c>
     </row>
     <row r="37" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D37" s="5"/>
+      <c r="D37" s="4"/>
       <c r="E37" t="s">
         <v>13</v>
       </c>
@@ -973,7 +1009,7 @@
       </c>
     </row>
     <row r="38" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D38" s="5"/>
+      <c r="D38" s="4"/>
       <c r="E38" t="s">
         <v>14</v>
       </c>
@@ -985,7 +1021,7 @@
       </c>
     </row>
     <row r="39" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D39" s="5"/>
+      <c r="D39" s="4"/>
       <c r="E39" t="s">
         <v>15</v>
       </c>
@@ -997,13 +1033,119 @@
       </c>
     </row>
     <row r="40" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="4">
+        <v>5</v>
+      </c>
+      <c r="E41" t="s">
+        <v>9</v>
+      </c>
+      <c r="F41">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G41">
+        <v>847.86075000000005</v>
+      </c>
+    </row>
+    <row r="42" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="4"/>
+      <c r="E42" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G42">
+        <v>838.84561099999996</v>
+      </c>
+    </row>
+    <row r="43" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="4"/>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G43">
+        <v>853.22697500000004</v>
+      </c>
+    </row>
+    <row r="44" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D44" s="4"/>
+      <c r="E44" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G44">
+        <v>837.32505200000003</v>
+      </c>
+    </row>
+    <row r="45" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D45" s="4"/>
+      <c r="E45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45">
+        <v>0.58333299999999999</v>
+      </c>
+      <c r="G45">
+        <v>843.81196799999998</v>
+      </c>
+    </row>
+    <row r="46" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D46" s="4"/>
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46">
+        <v>0.66666700000000001</v>
+      </c>
+      <c r="G46">
+        <v>1067.962276</v>
+      </c>
+    </row>
+    <row r="47" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D47" s="4"/>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G47">
+        <v>858.89092200000005</v>
+      </c>
+    </row>
+    <row r="48" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D48" s="4"/>
+      <c r="E48" t="s">
+        <v>15</v>
+      </c>
+      <c r="F48">
+        <v>0.54166700000000001</v>
+      </c>
+      <c r="G48">
+        <v>855.25156200000004</v>
+      </c>
+    </row>
+    <row r="49" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D41:D48"/>
+    <mergeCell ref="D49:G49"/>
     <mergeCell ref="D32:D39"/>
     <mergeCell ref="D40:G40"/>
     <mergeCell ref="D31:G31"/>
@@ -1019,7 +1161,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9F3D6F7-9B83-4803-A2A9-5F6E3F05FBE9}">
-  <dimension ref="D4:G40"/>
+  <dimension ref="D4:G49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="13.21875" customWidth="1"/>
@@ -1041,7 +1183,7 @@
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
       <c r="E5" t="s">
@@ -1055,7 +1197,7 @@
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D6" s="5"/>
+      <c r="D6" s="4"/>
       <c r="E6" t="s">
         <v>16</v>
       </c>
@@ -1067,7 +1209,7 @@
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D7" s="5"/>
+      <c r="D7" s="4"/>
       <c r="E7" t="s">
         <v>10</v>
       </c>
@@ -1079,7 +1221,7 @@
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D8" s="5"/>
+      <c r="D8" s="4"/>
       <c r="E8" t="s">
         <v>11</v>
       </c>
@@ -1091,7 +1233,7 @@
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D9" s="5"/>
+      <c r="D9" s="4"/>
       <c r="E9" t="s">
         <v>12</v>
       </c>
@@ -1103,7 +1245,7 @@
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D10" s="5"/>
+      <c r="D10" s="4"/>
       <c r="E10" t="s">
         <v>13</v>
       </c>
@@ -1115,7 +1257,7 @@
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D11" s="5"/>
+      <c r="D11" s="4"/>
       <c r="E11" t="s">
         <v>14</v>
       </c>
@@ -1127,7 +1269,7 @@
       </c>
     </row>
     <row r="12" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D12" s="5"/>
+      <c r="D12" s="4"/>
       <c r="E12" t="s">
         <v>15</v>
       </c>
@@ -1139,13 +1281,13 @@
       </c>
     </row>
     <row r="13" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>2</v>
       </c>
       <c r="E14" t="s">
@@ -1159,7 +1301,7 @@
       </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D15" s="5"/>
+      <c r="D15" s="4"/>
       <c r="E15" t="s">
         <v>16</v>
       </c>
@@ -1171,7 +1313,7 @@
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D16" s="5"/>
+      <c r="D16" s="4"/>
       <c r="E16" t="s">
         <v>10</v>
       </c>
@@ -1183,7 +1325,7 @@
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D17" s="5"/>
+      <c r="D17" s="4"/>
       <c r="E17" t="s">
         <v>11</v>
       </c>
@@ -1195,7 +1337,7 @@
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D18" s="5"/>
+      <c r="D18" s="4"/>
       <c r="E18" t="s">
         <v>12</v>
       </c>
@@ -1207,7 +1349,7 @@
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="5"/>
+      <c r="D19" s="4"/>
       <c r="E19" s="3" t="s">
         <v>13</v>
       </c>
@@ -1219,7 +1361,7 @@
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D20" s="5"/>
+      <c r="D20" s="4"/>
       <c r="E20" t="s">
         <v>14</v>
       </c>
@@ -1231,7 +1373,7 @@
       </c>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D21" s="5"/>
+      <c r="D21" s="4"/>
       <c r="E21" t="s">
         <v>15</v>
       </c>
@@ -1243,13 +1385,13 @@
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D23" s="5">
+      <c r="D23" s="4">
         <v>3</v>
       </c>
       <c r="E23" t="s">
@@ -1263,7 +1405,7 @@
       </c>
     </row>
     <row r="24" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D24" s="5"/>
+      <c r="D24" s="4"/>
       <c r="E24" t="s">
         <v>16</v>
       </c>
@@ -1275,7 +1417,7 @@
       </c>
     </row>
     <row r="25" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D25" s="5"/>
+      <c r="D25" s="4"/>
       <c r="E25" t="s">
         <v>10</v>
       </c>
@@ -1287,7 +1429,7 @@
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D26" s="5"/>
+      <c r="D26" s="4"/>
       <c r="E26" t="s">
         <v>11</v>
       </c>
@@ -1299,7 +1441,7 @@
       </c>
     </row>
     <row r="27" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D27" s="5"/>
+      <c r="D27" s="4"/>
       <c r="E27" t="s">
         <v>12</v>
       </c>
@@ -1311,7 +1453,7 @@
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D28" s="5"/>
+      <c r="D28" s="4"/>
       <c r="E28" t="s">
         <v>13</v>
       </c>
@@ -1323,7 +1465,7 @@
       </c>
     </row>
     <row r="29" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D29" s="5"/>
+      <c r="D29" s="4"/>
       <c r="E29" t="s">
         <v>14</v>
       </c>
@@ -1335,7 +1477,7 @@
       </c>
     </row>
     <row r="30" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D30" s="5"/>
+      <c r="D30" s="4"/>
       <c r="E30" t="s">
         <v>15</v>
       </c>
@@ -1347,13 +1489,13 @@
       </c>
     </row>
     <row r="31" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
+      <c r="D31" s="5"/>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5"/>
+      <c r="G31" s="5"/>
     </row>
     <row r="32" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D32" s="5">
+      <c r="D32" s="4">
         <v>4</v>
       </c>
       <c r="E32" t="s">
@@ -1367,7 +1509,7 @@
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D33" s="5"/>
+      <c r="D33" s="4"/>
       <c r="E33" t="s">
         <v>16</v>
       </c>
@@ -1379,7 +1521,7 @@
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D34" s="5"/>
+      <c r="D34" s="4"/>
       <c r="E34" t="s">
         <v>10</v>
       </c>
@@ -1391,7 +1533,7 @@
       </c>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D35" s="5"/>
+      <c r="D35" s="4"/>
       <c r="E35" t="s">
         <v>11</v>
       </c>
@@ -1403,7 +1545,7 @@
       </c>
     </row>
     <row r="36" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D36" s="5"/>
+      <c r="D36" s="4"/>
       <c r="E36" t="s">
         <v>12</v>
       </c>
@@ -1415,7 +1557,7 @@
       </c>
     </row>
     <row r="37" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D37" s="5"/>
+      <c r="D37" s="4"/>
       <c r="E37" t="s">
         <v>13</v>
       </c>
@@ -1427,7 +1569,7 @@
       </c>
     </row>
     <row r="38" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D38" s="5"/>
+      <c r="D38" s="4"/>
       <c r="E38" t="s">
         <v>14</v>
       </c>
@@ -1439,7 +1581,7 @@
       </c>
     </row>
     <row r="39" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D39" s="5"/>
+      <c r="D39" s="4"/>
       <c r="E39" t="s">
         <v>15</v>
       </c>
@@ -1451,13 +1593,119 @@
       </c>
     </row>
     <row r="40" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D40" s="4"/>
-      <c r="E40" s="4"/>
-      <c r="F40" s="4"/>
-      <c r="G40" s="4"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+      <c r="G40" s="5"/>
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="4">
+        <v>5</v>
+      </c>
+      <c r="E41" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" s="2">
+        <v>0.91666700000000001</v>
+      </c>
+      <c r="G41" s="2">
+        <v>937.70045300000004</v>
+      </c>
+    </row>
+    <row r="42" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="4"/>
+      <c r="E42" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" s="2">
+        <v>0.91666700000000001</v>
+      </c>
+      <c r="G42" s="2">
+        <v>936.699343</v>
+      </c>
+    </row>
+    <row r="43" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="4"/>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="G43" s="2">
+        <v>931.72322299999996</v>
+      </c>
+    </row>
+    <row r="44" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D44" s="4"/>
+      <c r="E44" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="G44" s="2">
+        <v>907.72775799999999</v>
+      </c>
+    </row>
+    <row r="45" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D45" s="4"/>
+      <c r="E45" t="s">
+        <v>12</v>
+      </c>
+      <c r="F45" s="2">
+        <v>0.91666700000000001</v>
+      </c>
+      <c r="G45" s="2">
+        <v>936.01575700000001</v>
+      </c>
+    </row>
+    <row r="46" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D46" s="4"/>
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" s="2">
+        <v>0.875</v>
+      </c>
+      <c r="G46" s="2">
+        <v>1101.727549</v>
+      </c>
+    </row>
+    <row r="47" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D47" s="4"/>
+      <c r="E47" t="s">
+        <v>14</v>
+      </c>
+      <c r="F47" s="2">
+        <v>0.91666700000000001</v>
+      </c>
+      <c r="G47" s="2">
+        <v>940.72508100000005</v>
+      </c>
+    </row>
+    <row r="48" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D48" s="4"/>
+      <c r="E48" t="s">
+        <v>15</v>
+      </c>
+      <c r="F48" s="2">
+        <v>0.91666700000000001</v>
+      </c>
+      <c r="G48" s="2">
+        <v>933.69020699999999</v>
+      </c>
+    </row>
+    <row r="49" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+      <c r="G49" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D41:D48"/>
+    <mergeCell ref="D49:G49"/>
     <mergeCell ref="D32:D39"/>
     <mergeCell ref="D40:G40"/>
     <mergeCell ref="D31:G31"/>
@@ -1473,7 +1721,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9B1F934-9143-4061-8956-2969F906ECCB}">
-  <dimension ref="D4:G36"/>
+  <dimension ref="D4:G44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="16.33203125" customWidth="1"/>
@@ -1495,7 +1743,7 @@
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
       <c r="E5" t="s">
@@ -1509,7 +1757,7 @@
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D6" s="5"/>
+      <c r="D6" s="4"/>
       <c r="E6" t="s">
         <v>10</v>
       </c>
@@ -1521,7 +1769,7 @@
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D7" s="5"/>
+      <c r="D7" s="4"/>
       <c r="E7" t="s">
         <v>11</v>
       </c>
@@ -1533,7 +1781,7 @@
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D8" s="5"/>
+      <c r="D8" s="4"/>
       <c r="E8" t="s">
         <v>12</v>
       </c>
@@ -1545,7 +1793,7 @@
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D9" s="5"/>
+      <c r="D9" s="4"/>
       <c r="E9" t="s">
         <v>13</v>
       </c>
@@ -1557,7 +1805,7 @@
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D10" s="5"/>
+      <c r="D10" s="4"/>
       <c r="E10" t="s">
         <v>14</v>
       </c>
@@ -1569,7 +1817,7 @@
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D11" s="5"/>
+      <c r="D11" s="4"/>
       <c r="E11" t="s">
         <v>15</v>
       </c>
@@ -1587,7 +1835,7 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>2</v>
       </c>
       <c r="E13" t="s">
@@ -1601,7 +1849,7 @@
       </c>
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D14" s="5"/>
+      <c r="D14" s="4"/>
       <c r="E14" t="s">
         <v>10</v>
       </c>
@@ -1613,7 +1861,7 @@
       </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D15" s="5"/>
+      <c r="D15" s="4"/>
       <c r="E15" t="s">
         <v>11</v>
       </c>
@@ -1625,7 +1873,7 @@
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D16" s="5"/>
+      <c r="D16" s="4"/>
       <c r="E16" t="s">
         <v>12</v>
       </c>
@@ -1637,7 +1885,7 @@
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D17" s="5"/>
+      <c r="D17" s="4"/>
       <c r="E17" t="s">
         <v>13</v>
       </c>
@@ -1649,7 +1897,7 @@
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D18" s="5"/>
+      <c r="D18" s="4"/>
       <c r="E18" t="s">
         <v>14</v>
       </c>
@@ -1661,7 +1909,7 @@
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="5"/>
+      <c r="D19" s="4"/>
       <c r="E19" t="s">
         <v>15</v>
       </c>
@@ -1673,13 +1921,13 @@
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>3</v>
       </c>
       <c r="E21" t="s">
@@ -1693,7 +1941,7 @@
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D22" s="5"/>
+      <c r="D22" s="4"/>
       <c r="E22" t="s">
         <v>10</v>
       </c>
@@ -1705,7 +1953,7 @@
       </c>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D23" s="5"/>
+      <c r="D23" s="4"/>
       <c r="E23" t="s">
         <v>11</v>
       </c>
@@ -1717,7 +1965,7 @@
       </c>
     </row>
     <row r="24" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D24" s="5"/>
+      <c r="D24" s="4"/>
       <c r="E24" t="s">
         <v>12</v>
       </c>
@@ -1729,7 +1977,7 @@
       </c>
     </row>
     <row r="25" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D25" s="5"/>
+      <c r="D25" s="4"/>
       <c r="E25" t="s">
         <v>13</v>
       </c>
@@ -1741,7 +1989,7 @@
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D26" s="5"/>
+      <c r="D26" s="4"/>
       <c r="E26" t="s">
         <v>14</v>
       </c>
@@ -1753,7 +2001,7 @@
       </c>
     </row>
     <row r="27" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D27" s="5"/>
+      <c r="D27" s="4"/>
       <c r="E27" t="s">
         <v>15</v>
       </c>
@@ -1765,13 +2013,13 @@
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
     </row>
     <row r="29" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D29" s="5">
+      <c r="D29" s="4">
         <v>4</v>
       </c>
       <c r="E29" t="s">
@@ -1785,7 +2033,7 @@
       </c>
     </row>
     <row r="30" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D30" s="5"/>
+      <c r="D30" s="4"/>
       <c r="E30" t="s">
         <v>10</v>
       </c>
@@ -1797,7 +2045,7 @@
       </c>
     </row>
     <row r="31" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D31" s="5"/>
+      <c r="D31" s="4"/>
       <c r="E31" t="s">
         <v>11</v>
       </c>
@@ -1809,7 +2057,7 @@
       </c>
     </row>
     <row r="32" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D32" s="5"/>
+      <c r="D32" s="4"/>
       <c r="E32" t="s">
         <v>12</v>
       </c>
@@ -1821,7 +2069,7 @@
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D33" s="5"/>
+      <c r="D33" s="4"/>
       <c r="E33" t="s">
         <v>13</v>
       </c>
@@ -1833,7 +2081,7 @@
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D34" s="5"/>
+      <c r="D34" s="4"/>
       <c r="E34" t="s">
         <v>14</v>
       </c>
@@ -1845,7 +2093,7 @@
       </c>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D35" s="5"/>
+      <c r="D35" s="4"/>
       <c r="E35" t="s">
         <v>15</v>
       </c>
@@ -1857,13 +2105,107 @@
       </c>
     </row>
     <row r="36" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D37" s="4">
+        <v>5</v>
+      </c>
+      <c r="E37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37">
+        <v>0.29166700000000001</v>
+      </c>
+      <c r="G37">
+        <v>297.578644</v>
+      </c>
+    </row>
+    <row r="38" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D38" s="4"/>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38">
+        <v>0.16666700000000001</v>
+      </c>
+      <c r="G38">
+        <v>196.72213500000001</v>
+      </c>
+    </row>
+    <row r="39" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D39" s="4"/>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39">
+        <v>0.125</v>
+      </c>
+      <c r="G39">
+        <v>116.041706</v>
+      </c>
+    </row>
+    <row r="40" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D40" s="4"/>
+      <c r="E40" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40">
+        <v>0.125</v>
+      </c>
+      <c r="G40">
+        <v>102.865477</v>
+      </c>
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="4"/>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41">
+        <v>0.25</v>
+      </c>
+      <c r="G41">
+        <v>275.98971899999998</v>
+      </c>
+    </row>
+    <row r="42" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="4"/>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42">
+        <v>0</v>
+      </c>
+      <c r="G42">
+        <v>6.3266600000000004</v>
+      </c>
+    </row>
+    <row r="43" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="4"/>
+      <c r="E43" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43">
+        <v>0.25</v>
+      </c>
+      <c r="G43">
+        <v>292.207177</v>
+      </c>
+    </row>
+    <row r="44" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D37:D43"/>
+    <mergeCell ref="D44:G44"/>
     <mergeCell ref="D29:D35"/>
     <mergeCell ref="D36:G36"/>
     <mergeCell ref="D28:G28"/>
@@ -1879,7 +2221,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA9C7C1F-8E69-4E9D-9311-55B2096F876D}">
-  <dimension ref="D4:G36"/>
+  <dimension ref="D4:G44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="16.33203125" customWidth="1"/>
@@ -1901,7 +2243,7 @@
       </c>
     </row>
     <row r="5" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1</v>
       </c>
       <c r="E5" t="s">
@@ -1915,7 +2257,7 @@
       </c>
     </row>
     <row r="6" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D6" s="5"/>
+      <c r="D6" s="4"/>
       <c r="E6" t="s">
         <v>10</v>
       </c>
@@ -1927,7 +2269,7 @@
       </c>
     </row>
     <row r="7" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D7" s="5"/>
+      <c r="D7" s="4"/>
       <c r="E7" t="s">
         <v>11</v>
       </c>
@@ -1939,7 +2281,7 @@
       </c>
     </row>
     <row r="8" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D8" s="5"/>
+      <c r="D8" s="4"/>
       <c r="E8" t="s">
         <v>12</v>
       </c>
@@ -1951,7 +2293,7 @@
       </c>
     </row>
     <row r="9" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D9" s="5"/>
+      <c r="D9" s="4"/>
       <c r="E9" t="s">
         <v>13</v>
       </c>
@@ -1963,7 +2305,7 @@
       </c>
     </row>
     <row r="10" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D10" s="5"/>
+      <c r="D10" s="4"/>
       <c r="E10" t="s">
         <v>14</v>
       </c>
@@ -1975,7 +2317,7 @@
       </c>
     </row>
     <row r="11" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D11" s="5"/>
+      <c r="D11" s="4"/>
       <c r="E11" t="s">
         <v>15</v>
       </c>
@@ -1993,7 +2335,7 @@
       <c r="G12" s="6"/>
     </row>
     <row r="13" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>2</v>
       </c>
       <c r="E13" t="s">
@@ -2007,7 +2349,7 @@
       </c>
     </row>
     <row r="14" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D14" s="5"/>
+      <c r="D14" s="4"/>
       <c r="E14" t="s">
         <v>10</v>
       </c>
@@ -2019,7 +2361,7 @@
       </c>
     </row>
     <row r="15" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D15" s="5"/>
+      <c r="D15" s="4"/>
       <c r="E15" t="s">
         <v>11</v>
       </c>
@@ -2031,7 +2373,7 @@
       </c>
     </row>
     <row r="16" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D16" s="5"/>
+      <c r="D16" s="4"/>
       <c r="E16" t="s">
         <v>12</v>
       </c>
@@ -2043,7 +2385,7 @@
       </c>
     </row>
     <row r="17" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D17" s="5"/>
+      <c r="D17" s="4"/>
       <c r="E17" t="s">
         <v>13</v>
       </c>
@@ -2055,7 +2397,7 @@
       </c>
     </row>
     <row r="18" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D18" s="5"/>
+      <c r="D18" s="4"/>
       <c r="E18" t="s">
         <v>14</v>
       </c>
@@ -2067,7 +2409,7 @@
       </c>
     </row>
     <row r="19" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D19" s="5"/>
+      <c r="D19" s="4"/>
       <c r="E19" t="s">
         <v>15</v>
       </c>
@@ -2079,13 +2421,13 @@
       </c>
     </row>
     <row r="20" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
     </row>
     <row r="21" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D21" s="5">
+      <c r="D21" s="4">
         <v>3</v>
       </c>
       <c r="E21" t="s">
@@ -2099,7 +2441,7 @@
       </c>
     </row>
     <row r="22" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D22" s="5"/>
+      <c r="D22" s="4"/>
       <c r="E22" t="s">
         <v>10</v>
       </c>
@@ -2111,7 +2453,7 @@
       </c>
     </row>
     <row r="23" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D23" s="5"/>
+      <c r="D23" s="4"/>
       <c r="E23" t="s">
         <v>11</v>
       </c>
@@ -2123,7 +2465,7 @@
       </c>
     </row>
     <row r="24" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D24" s="5"/>
+      <c r="D24" s="4"/>
       <c r="E24" t="s">
         <v>12</v>
       </c>
@@ -2135,7 +2477,7 @@
       </c>
     </row>
     <row r="25" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D25" s="5"/>
+      <c r="D25" s="4"/>
       <c r="E25" t="s">
         <v>13</v>
       </c>
@@ -2147,7 +2489,7 @@
       </c>
     </row>
     <row r="26" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D26" s="5"/>
+      <c r="D26" s="4"/>
       <c r="E26" t="s">
         <v>14</v>
       </c>
@@ -2159,7 +2501,7 @@
       </c>
     </row>
     <row r="27" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D27" s="5"/>
+      <c r="D27" s="4"/>
       <c r="E27" t="s">
         <v>15</v>
       </c>
@@ -2171,13 +2513,13 @@
       </c>
     </row>
     <row r="28" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
     </row>
     <row r="29" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D29" s="5">
+      <c r="D29" s="4">
         <v>4</v>
       </c>
       <c r="E29" t="s">
@@ -2191,7 +2533,7 @@
       </c>
     </row>
     <row r="30" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D30" s="5"/>
+      <c r="D30" s="4"/>
       <c r="E30" t="s">
         <v>10</v>
       </c>
@@ -2203,7 +2545,7 @@
       </c>
     </row>
     <row r="31" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D31" s="5"/>
+      <c r="D31" s="4"/>
       <c r="E31" t="s">
         <v>11</v>
       </c>
@@ -2215,7 +2557,7 @@
       </c>
     </row>
     <row r="32" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D32" s="5"/>
+      <c r="D32" s="4"/>
       <c r="E32" t="s">
         <v>12</v>
       </c>
@@ -2227,7 +2569,7 @@
       </c>
     </row>
     <row r="33" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D33" s="5"/>
+      <c r="D33" s="4"/>
       <c r="E33" t="s">
         <v>13</v>
       </c>
@@ -2239,7 +2581,7 @@
       </c>
     </row>
     <row r="34" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D34" s="5"/>
+      <c r="D34" s="4"/>
       <c r="E34" t="s">
         <v>14</v>
       </c>
@@ -2251,7 +2593,7 @@
       </c>
     </row>
     <row r="35" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D35" s="5"/>
+      <c r="D35" s="4"/>
       <c r="E35" t="s">
         <v>15</v>
       </c>
@@ -2263,13 +2605,107 @@
       </c>
     </row>
     <row r="36" spans="4:7" x14ac:dyDescent="0.3">
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
+      <c r="D36" s="5"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="5"/>
+    </row>
+    <row r="37" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D37" s="4">
+        <v>5</v>
+      </c>
+      <c r="E37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F37">
+        <v>8.3333000000000004E-2</v>
+      </c>
+      <c r="G37">
+        <v>95.155683999999994</v>
+      </c>
+    </row>
+    <row r="38" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D38" s="4"/>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38">
+        <v>8.3333000000000004E-2</v>
+      </c>
+      <c r="G38">
+        <v>91.139943000000002</v>
+      </c>
+    </row>
+    <row r="39" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D39" s="4"/>
+      <c r="E39" t="s">
+        <v>11</v>
+      </c>
+      <c r="F39">
+        <v>8.3333000000000004E-2</v>
+      </c>
+      <c r="G39">
+        <v>50.897694999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D40" s="4"/>
+      <c r="E40" t="s">
+        <v>12</v>
+      </c>
+      <c r="F40">
+        <v>4.1667000000000003E-2</v>
+      </c>
+      <c r="G40">
+        <v>45.668508000000003</v>
+      </c>
+    </row>
+    <row r="41" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D41" s="4"/>
+      <c r="E41" t="s">
+        <v>13</v>
+      </c>
+      <c r="F41">
+        <v>4.1667000000000003E-2</v>
+      </c>
+      <c r="G41">
+        <v>61.417313999999998</v>
+      </c>
+    </row>
+    <row r="42" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D42" s="4"/>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42">
+        <v>4.1667000000000003E-2</v>
+      </c>
+      <c r="G42">
+        <v>8.7120560000000005</v>
+      </c>
+    </row>
+    <row r="43" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D43" s="4"/>
+      <c r="E43" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43">
+        <v>8.3333000000000004E-2</v>
+      </c>
+      <c r="G43">
+        <v>89.088755000000006</v>
+      </c>
+    </row>
+    <row r="44" spans="4:7" x14ac:dyDescent="0.3">
+      <c r="D44" s="5"/>
+      <c r="E44" s="5"/>
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
+    <mergeCell ref="D37:D43"/>
+    <mergeCell ref="D44:G44"/>
     <mergeCell ref="D29:D35"/>
     <mergeCell ref="D36:G36"/>
     <mergeCell ref="D28:G28"/>

</xml_diff>